<commit_message>
Actualizacao dos dados e daa pagina dos indicadores
</commit_message>
<xml_diff>
--- a/Financeiro_Report.xlsx
+++ b/Financeiro_Report.xlsx
@@ -43226,13 +43226,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C7C9E419-2B15-4FF4-BA2A-B9C13C7D2381}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{61B6F950-EEDE-406E-AB5C-D1801BF046C5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5098AC2B-D7B0-4607-B22D-33F56A5AED91}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACB67815-060E-4D5C-BED0-DD003A67B1F8}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FED950E6-1082-4146-8221-413D8847245E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{795DA35A-FC45-4539-8709-3106F531B73B}"/>
 </file>
</xml_diff>